<commit_message>
Trainees work Live Watch, not picker cases (Options + Training roles)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/configuration-options.xlsx
+++ b/docs/configuration-options.xlsx
@@ -1122,21 +1122,21 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="84" customHeight="1">
+    <row r="37" ht="70" customHeight="1">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Should residents and fellows be assigned peer review cases?</t>
+          <t>How should residents and fellows take part in peer review?</t>
         </is>
       </c>
       <c r="B37" s="10" t="inlineStr">
         <is>
-          <t>No. Trainees are not assigned review cases or discrepant exams. To include an individual trainee in assigned review (for example, for a Graduate Medical Education quality improvement project), give them a reviewer role instead of the resident / fellow role.</t>
+          <t>Through Live Watch, not picker assignments. Trainees are not assigned picker cases or discrepant exams; they work the Live Watch page, claiming AI-flagged exams and submitting preliminary reviews that escalate directly to Quality Champions.</t>
         </is>
       </c>
       <c r="C37" s="11" t="n"/>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>Protect trainees from unsupervised discrepancy review while allowing structured participation where your program wants it.</t>
+          <t>Hands-on discrepancy review for trainees (for example, toward a Graduate Medical Education quality improvement project), with Quality Champions handling every escalation.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1">
+    <row r="17" ht="56" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
           <t>Residents and fellows</t>
@@ -1429,12 +1429,12 @@
       </c>
       <c r="B17" s="10" t="inlineStr">
         <is>
-          <t>Admin → Users and Admin → Roles</t>
+          <t>Admin → Roles and Admin → Users</t>
         </is>
       </c>
       <c r="C17" s="10" t="inlineStr">
         <is>
-          <t>Resident / fellow role ("Resident / fellow assignments") or a reviewer role</t>
+          <t>Give trainees a role with "Work Community Watch cases" and "Resident / fellow assignments" (no picker cases), then turn on Community Watch for each trainee in Admin → Users</t>
         </is>
       </c>
     </row>

</xml_diff>